<commit_message>
Prueba para actualizar el proyecto final
</commit_message>
<xml_diff>
--- a/data/Datos_Tabla_Mortalidad_CDMX.xlsx
+++ b/data/Datos_Tabla_Mortalidad_CDMX.xlsx
@@ -1,22 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Rafa\Proyecto final demografía\Demography_9219\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B350D20-A022-4B49-9CA9-25FB83A0F705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E611947E-0FD5-4598-9325-F82D547D5FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{45F953CB-AACF-024F-88B1-CE3D562CB5AD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="1" xr2:uid="{45F953CB-AACF-024F-88B1-CE3D562CB5AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabla de Mortalidad Mujeres" sheetId="1" r:id="rId1"/>
     <sheet name="Tabla de Mortalidad Hombres " sheetId="2" r:id="rId2"/>
-    <sheet name="Mujeres" sheetId="3" r:id="rId3"/>
-    <sheet name="Hombres" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
   <si>
     <t xml:space="preserve">Tabla de Mortalidad mujeres </t>
   </si>
@@ -90,7 +88,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -103,6 +101,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -112,7 +116,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -135,11 +139,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -151,7 +170,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -486,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43BD4C73-3377-1D49-9902-8ABC9947BCB4}">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -494,7 +521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -535,19 +562,18 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>0</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
-        <f>D4/Mujeres!A3</f>
-        <v>41159.242598785168</v>
-      </c>
-      <c r="D4" s="5">
-        <v>39014</v>
+      <c r="C4" s="6">
+        <v>85241</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1480</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -559,19 +585,18 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="2">
         <v>4</v>
       </c>
-      <c r="C5" s="3">
-        <f>D5/Mujeres!A4</f>
-        <v>200150.36259921559</v>
-      </c>
-      <c r="D5" s="5">
-        <v>5150</v>
+      <c r="C5" s="6">
+        <v>358620</v>
+      </c>
+      <c r="D5" s="6">
+        <v>240</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -583,19 +608,18 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
       </c>
-      <c r="C6" s="3">
-        <f>D6/Mujeres!A5</f>
-        <v>281464.21899999998</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2697</v>
+      <c r="C6" s="6">
+        <v>468145</v>
+      </c>
+      <c r="D6" s="6">
+        <v>165</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -607,19 +631,18 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>10</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
       </c>
-      <c r="C7" s="3">
-        <f>D7/Mujeres!A6</f>
-        <v>302383.62900000002</v>
-      </c>
-      <c r="D7" s="5">
-        <v>2946</v>
+      <c r="C7" s="6">
+        <v>490312</v>
+      </c>
+      <c r="D7" s="6">
+        <v>155</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -631,19 +654,18 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>15</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
       </c>
-      <c r="C8" s="3">
-        <f>D8/Mujeres!A7</f>
-        <v>322888.02600000001</v>
-      </c>
-      <c r="D8" s="5">
-        <v>5659</v>
+      <c r="C8" s="6">
+        <v>512987</v>
+      </c>
+      <c r="D8" s="6">
+        <v>320</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -655,19 +677,18 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>20</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
       </c>
-      <c r="C9" s="3">
-        <f>D9/Mujeres!A8</f>
-        <v>358243.18599999999</v>
-      </c>
-      <c r="D9" s="5">
-        <v>7332</v>
+      <c r="C9" s="6">
+        <v>535423</v>
+      </c>
+      <c r="D9" s="6">
+        <v>410</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -679,19 +700,18 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>25</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
       </c>
-      <c r="C10" s="3">
-        <f>D10/Mujeres!A9</f>
-        <v>380688.283</v>
-      </c>
-      <c r="D10" s="5">
-        <v>8554</v>
+      <c r="C10" s="6">
+        <v>556198</v>
+      </c>
+      <c r="D10" s="6">
+        <v>510</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -703,19 +723,18 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>30</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
       </c>
-      <c r="C11" s="3">
-        <f>D11/Mujeres!A10</f>
-        <v>380119.34899999999</v>
-      </c>
-      <c r="D11" s="5">
-        <v>10557</v>
+      <c r="C11" s="6">
+        <v>572345</v>
+      </c>
+      <c r="D11" s="6">
+        <v>680</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -727,19 +746,18 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>35</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
       </c>
-      <c r="C12" s="3">
-        <f>D12/Mujeres!A11</f>
-        <v>367296.37900000002</v>
-      </c>
-      <c r="D12" s="5">
-        <v>14259</v>
+      <c r="C12" s="6">
+        <v>585671</v>
+      </c>
+      <c r="D12" s="6">
+        <v>920</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -751,19 +769,18 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>40</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
       </c>
-      <c r="C13" s="3">
-        <f>D13/Mujeres!A12</f>
-        <v>352496.565</v>
-      </c>
-      <c r="D13" s="5">
-        <v>19836</v>
+      <c r="C13" s="6">
+        <v>598124</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1350</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -775,19 +792,18 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>45</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
       </c>
-      <c r="C14" s="3">
-        <f>D14/Mujeres!A13</f>
-        <v>351613.3</v>
-      </c>
-      <c r="D14" s="5">
-        <v>29202</v>
+      <c r="C14" s="6">
+        <v>601452</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1890</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -799,19 +815,18 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>50</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
       </c>
-      <c r="C15" s="3">
-        <f>D15/Mujeres!A14</f>
-        <v>333069.23800000001</v>
-      </c>
-      <c r="D15" s="5">
-        <v>40024</v>
+      <c r="C15" s="6">
+        <v>588903</v>
+      </c>
+      <c r="D15" s="6">
+        <v>2650</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -823,19 +838,18 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>55</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
       </c>
-      <c r="C16" s="3">
-        <f>D16/Mujeres!A15</f>
-        <v>281391.136</v>
-      </c>
-      <c r="D16" s="5">
-        <v>53150</v>
+      <c r="C16" s="6">
+        <v>552341</v>
+      </c>
+      <c r="D16" s="6">
+        <v>3420</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -847,19 +861,18 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>60</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
       </c>
-      <c r="C17" s="3">
-        <f>D17/Mujeres!A16</f>
-        <v>253658.04199999999</v>
-      </c>
-      <c r="D17" s="5">
-        <v>68338</v>
+      <c r="C17" s="6">
+        <v>489678</v>
+      </c>
+      <c r="D17" s="6">
+        <v>4850</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -871,19 +884,18 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>65</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
       </c>
-      <c r="C18" s="3">
-        <f>D18/Mujeres!A17</f>
-        <v>193140.62899999999</v>
-      </c>
-      <c r="D18" s="5">
-        <v>82804</v>
+      <c r="C18" s="6">
+        <v>402156</v>
+      </c>
+      <c r="D18" s="6">
+        <v>6320</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -895,19 +907,18 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>70</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
       </c>
-      <c r="C19" s="3">
-        <f>D19/Mujeres!A18</f>
-        <v>148810.791</v>
-      </c>
-      <c r="D19" s="5">
-        <v>95186</v>
+      <c r="C19" s="6">
+        <v>315892</v>
+      </c>
+      <c r="D19" s="6">
+        <v>8950</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -919,19 +930,18 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>75</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
       </c>
-      <c r="C20" s="3">
-        <f>D20/Mujeres!A19</f>
-        <v>98970.747299999988</v>
-      </c>
-      <c r="D20" s="5">
-        <v>106789</v>
+      <c r="C20" s="6">
+        <v>224567</v>
+      </c>
+      <c r="D20" s="6">
+        <v>10850</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -943,19 +953,18 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>80</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
       </c>
-      <c r="C21" s="3">
-        <f>D21/Mujeres!A20</f>
-        <v>70046.554099999994</v>
-      </c>
-      <c r="D21" s="5">
-        <v>115310</v>
+      <c r="C21" s="6">
+        <v>134789</v>
+      </c>
+      <c r="D21" s="6">
+        <v>11200</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -967,17 +976,16 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>85</v>
       </c>
       <c r="B22" s="2"/>
-      <c r="C22" s="3">
-        <f>D22/Mujeres!A21</f>
-        <v>67061.372099999993</v>
-      </c>
-      <c r="D22" s="5">
-        <v>226406</v>
+      <c r="C22" s="6">
+        <v>115234</v>
+      </c>
+      <c r="D22" s="6">
+        <v>18500</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -988,6 +996,9 @@
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1004,7 +1015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1045,19 +1056,18 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>0</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
-        <f>D4/Hombres!A3</f>
-        <v>42317.937985787707</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50449</v>
+      <c r="C4" s="7">
+        <v>88412</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1850</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -1069,19 +1079,18 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="2">
         <v>4</v>
       </c>
-      <c r="C5" s="3">
-        <f>D5/Hombres!A4</f>
-        <v>205156.40142936358</v>
-      </c>
-      <c r="D5" s="5">
-        <v>6196</v>
+      <c r="C5" s="7">
+        <v>365240</v>
+      </c>
+      <c r="D5" s="6">
+        <v>310</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -1093,19 +1102,18 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
       </c>
-      <c r="C6" s="3">
-        <f>D6/Hombres!A5</f>
-        <v>290343.92700000003</v>
-      </c>
-      <c r="D6" s="5">
-        <v>3234</v>
+      <c r="C6" s="7">
+        <v>472156</v>
+      </c>
+      <c r="D6" s="6">
+        <v>210</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -1117,19 +1125,18 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>10</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
       </c>
-      <c r="C7" s="3">
-        <f>D7/Hombres!A6</f>
-        <v>311772.05499999999</v>
-      </c>
-      <c r="D7" s="5">
-        <v>3988</v>
+      <c r="C7" s="7">
+        <v>496210</v>
+      </c>
+      <c r="D7" s="6">
+        <v>205</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -1141,19 +1148,18 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>15</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
       </c>
-      <c r="C8" s="3">
-        <f>D8/Hombres!A7</f>
-        <v>334250.92099999997</v>
-      </c>
-      <c r="D8" s="5">
-        <v>12474</v>
+      <c r="C8" s="7">
+        <v>508412</v>
+      </c>
+      <c r="D8" s="6">
+        <v>680</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -1165,19 +1171,18 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>20</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
       </c>
-      <c r="C9" s="3">
-        <f>D9/Hombres!A8</f>
-        <v>360980.01400000002</v>
-      </c>
-      <c r="D9" s="5">
-        <v>21116</v>
+      <c r="C9" s="7">
+        <v>521345</v>
+      </c>
+      <c r="D9" s="6">
+        <v>920</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -1189,19 +1194,18 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>25</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
       </c>
-      <c r="C10" s="3">
-        <f>D10/Hombres!A9</f>
-        <v>371670.93900000001</v>
-      </c>
-      <c r="D10" s="5">
-        <v>25764</v>
+      <c r="C10" s="7">
+        <v>540112</v>
+      </c>
+      <c r="D10" s="7">
+        <v>1050</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -1213,19 +1217,18 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>30</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
       </c>
-      <c r="C11" s="3">
-        <f>D11/Hombres!A10</f>
-        <v>362367.95400000003</v>
-      </c>
-      <c r="D11" s="5">
-        <v>30175</v>
+      <c r="C11" s="7">
+        <v>555234</v>
+      </c>
+      <c r="D11" s="7">
+        <v>1280</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -1237,19 +1240,18 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>35</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
       </c>
-      <c r="C12" s="3">
-        <f>D12/Hombres!A11</f>
-        <v>341569.02500000002</v>
-      </c>
-      <c r="D12" s="5">
-        <v>35522</v>
+      <c r="C12" s="7">
+        <v>570412</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1650</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -1261,19 +1263,18 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>40</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
       </c>
-      <c r="C13" s="3">
-        <f>D13/Hombres!A12</f>
-        <v>316510.489</v>
-      </c>
-      <c r="D13" s="5">
-        <v>41456</v>
+      <c r="C13" s="7">
+        <v>582341</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2210</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1285,19 +1286,18 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>45</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
       </c>
-      <c r="C14" s="3">
-        <f>D14/Hombres!A13</f>
-        <v>310092.38799999998</v>
-      </c>
-      <c r="D14" s="5">
-        <v>51386</v>
+      <c r="C14" s="7">
+        <v>588903</v>
+      </c>
+      <c r="D14" s="7">
+        <v>2840</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1309,19 +1309,18 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>50</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
       </c>
-      <c r="C15" s="3">
-        <f>D15/Hombres!A14</f>
-        <v>282672.16399999999</v>
-      </c>
-      <c r="D15" s="5">
-        <v>62275</v>
+      <c r="C15" s="7">
+        <v>560112</v>
+      </c>
+      <c r="D15" s="7">
+        <v>3750</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -1333,19 +1332,18 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>55</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
       </c>
-      <c r="C16" s="3">
-        <f>D16/Hombres!A15</f>
-        <v>235278.02</v>
-      </c>
-      <c r="D16" s="5">
-        <v>74606</v>
+      <c r="C16" s="7">
+        <v>501456</v>
+      </c>
+      <c r="D16" s="7">
+        <v>4680</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -1357,19 +1355,18 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>60</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
       </c>
-      <c r="C17" s="3">
-        <f>D17/Hombres!A16</f>
-        <v>203731.67499999999</v>
-      </c>
-      <c r="D17" s="5">
-        <v>86957</v>
+      <c r="C17" s="7">
+        <v>415892</v>
+      </c>
+      <c r="D17" s="7">
+        <v>6250</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -1381,19 +1378,18 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>65</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
       </c>
-      <c r="C18" s="3">
-        <f>D18/Hombres!A17</f>
-        <v>152571.318</v>
-      </c>
-      <c r="D18" s="5">
-        <v>94843</v>
+      <c r="C18" s="7">
+        <v>321456</v>
+      </c>
+      <c r="D18" s="7">
+        <v>7820</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -1405,19 +1401,18 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>70</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
       </c>
-      <c r="C19" s="3">
-        <f>D19/Hombres!A18</f>
-        <v>111935.031</v>
-      </c>
-      <c r="D19" s="5">
-        <v>100787</v>
+      <c r="C19" s="7">
+        <v>225123</v>
+      </c>
+      <c r="D19" s="7">
+        <v>9410</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -1429,19 +1424,18 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>75</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
       </c>
-      <c r="C20" s="3">
-        <f>D20/Hombres!A19</f>
-        <v>72394.090599999996</v>
-      </c>
-      <c r="D20" s="5">
-        <v>100092</v>
+      <c r="C20" s="7">
+        <v>145678</v>
+      </c>
+      <c r="D20" s="7">
+        <v>9850</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1453,19 +1447,18 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>80</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
       </c>
-      <c r="C21" s="3">
-        <f>D21/Hombres!A20</f>
-        <v>45013.495300000002</v>
-      </c>
-      <c r="D21" s="5">
-        <v>91138</v>
+      <c r="C21" s="7">
+        <v>85412</v>
+      </c>
+      <c r="D21" s="7">
+        <v>9120</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -1477,17 +1470,16 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>85</v>
       </c>
       <c r="B22" s="3"/>
-      <c r="C22" s="3">
-        <f>D22/Hombres!A21</f>
-        <v>35718.739600000001</v>
-      </c>
-      <c r="D22" s="5">
-        <v>128221</v>
+      <c r="C22" s="7">
+        <v>62341</v>
+      </c>
+      <c r="D22" s="7">
+        <v>12450</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -1502,224 +1494,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A52C6FC-409A-4D0A-9423-9B089A1B462D}">
-  <dimension ref="A2:A21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>0.94787944424301707</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>2.5730655358903575E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>9.5820350081514266E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>9.7425909257805744E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>1.7526199624386195E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>2.0466544198275413E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>2.2469827367920331E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>2.7772856151029555E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>3.882150986301991E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>5.6272888786873712E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>8.3051465914400852E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
-        <v>0.12016720679560326</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
-        <v>0.18888299310181542</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>0.26940994837451282</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>0.42872388077394119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
-        <v>0.63964447309469652</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>1.0789955912558822</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>1.6461909009168521</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
-        <v>3.376101515823295</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9CFC32D-E305-4F8D-899E-272C2B6F92A2}">
-  <dimension ref="A2:A21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>1.1921422073292671</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>3.0201348614185528E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>1.1138514359213718E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>1.2791396586201416E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>3.7319268897392212E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>5.8496313316670212E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>6.9319382541232252E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>8.3271712266256293E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>0.10399654945292536</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>0.13097828173397438</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>0.1657119038987826</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
-        <v>0.22030821542088594</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
-        <v>0.31709719420454152</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>0.42682120980942218</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>0.62163060032030393</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
-        <v>0.90040623654269591</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>1.3825990377175896</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>2.0246816958468896</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
-        <v>3.5897403277914095</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>